<commit_message>
added deduplicate and trim nans
</commit_message>
<xml_diff>
--- a/scripts/golden_snapshot/visual_report.xlsx
+++ b/scripts/golden_snapshot/visual_report.xlsx
@@ -469,7 +469,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>4178</v>
+        <v>4166</v>
       </c>
     </row>
     <row r="3">
@@ -479,7 +479,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>4178</v>
+        <v>4166</v>
       </c>
     </row>
     <row r="4">
@@ -521,7 +521,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>3440.67</v>
+        <v>3451.03</v>
       </c>
     </row>
     <row r="8">
@@ -4052,7 +4052,7 @@
         <v>2319.2</v>
       </c>
       <c r="H11" t="n">
-        <v>52532.4</v>
+        <v>52532.39999999999</v>
       </c>
       <c r="I11" t="n">
         <v>12600.4</v>
@@ -5131,7 +5131,7 @@
         </is>
       </c>
       <c r="C57" t="n">
-        <v>52532.4</v>
+        <v>52532.39999999999</v>
       </c>
     </row>
     <row r="58">
@@ -5329,7 +5329,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S105"/>
+  <dimension ref="A1:S169"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11793,6 +11793,4050 @@
         <v>0</v>
       </c>
     </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Спортивное ориентирование</t>
+        </is>
+      </c>
+      <c r="B106" t="n">
+        <v>185</v>
+      </c>
+      <c r="C106" t="n">
+        <v>0</v>
+      </c>
+      <c r="D106" t="n">
+        <v>0</v>
+      </c>
+      <c r="E106" t="n">
+        <v>0</v>
+      </c>
+      <c r="F106" t="n">
+        <v>0</v>
+      </c>
+      <c r="G106" t="n">
+        <v>0</v>
+      </c>
+      <c r="H106" t="n">
+        <v>0</v>
+      </c>
+      <c r="I106" t="n">
+        <v>0</v>
+      </c>
+      <c r="J106" t="n">
+        <v>0</v>
+      </c>
+      <c r="K106" t="n">
+        <v>0</v>
+      </c>
+      <c r="L106" t="n">
+        <v>0</v>
+      </c>
+      <c r="M106" t="n">
+        <v>0</v>
+      </c>
+      <c r="N106" t="n">
+        <v>0</v>
+      </c>
+      <c r="O106" t="n">
+        <v>0</v>
+      </c>
+      <c r="P106" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q106" t="n">
+        <v>0</v>
+      </c>
+      <c r="R106" t="n">
+        <v>0</v>
+      </c>
+      <c r="S106" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Спортивный бридж</t>
+        </is>
+      </c>
+      <c r="B107" t="n">
+        <v>186</v>
+      </c>
+      <c r="C107" t="n">
+        <v>0</v>
+      </c>
+      <c r="D107" t="n">
+        <v>0</v>
+      </c>
+      <c r="E107" t="n">
+        <v>0</v>
+      </c>
+      <c r="F107" t="n">
+        <v>0</v>
+      </c>
+      <c r="G107" t="n">
+        <v>0</v>
+      </c>
+      <c r="H107" t="n">
+        <v>0</v>
+      </c>
+      <c r="I107" t="n">
+        <v>0</v>
+      </c>
+      <c r="J107" t="n">
+        <v>0</v>
+      </c>
+      <c r="K107" t="n">
+        <v>0</v>
+      </c>
+      <c r="L107" t="n">
+        <v>0</v>
+      </c>
+      <c r="M107" t="n">
+        <v>0</v>
+      </c>
+      <c r="N107" t="n">
+        <v>0</v>
+      </c>
+      <c r="O107" t="n">
+        <v>0</v>
+      </c>
+      <c r="P107" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q107" t="n">
+        <v>0</v>
+      </c>
+      <c r="R107" t="n">
+        <v>0</v>
+      </c>
+      <c r="S107" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Спортивный туризм - всего</t>
+        </is>
+      </c>
+      <c r="B108" t="n">
+        <v>187</v>
+      </c>
+      <c r="C108" t="n">
+        <v>0</v>
+      </c>
+      <c r="D108" t="n">
+        <v>0</v>
+      </c>
+      <c r="E108" t="n">
+        <v>0</v>
+      </c>
+      <c r="F108" t="n">
+        <v>0</v>
+      </c>
+      <c r="G108" t="n">
+        <v>0</v>
+      </c>
+      <c r="H108" t="n">
+        <v>0</v>
+      </c>
+      <c r="I108" t="n">
+        <v>0</v>
+      </c>
+      <c r="J108" t="n">
+        <v>0</v>
+      </c>
+      <c r="K108" t="n">
+        <v>0</v>
+      </c>
+      <c r="L108" t="n">
+        <v>0</v>
+      </c>
+      <c r="M108" t="n">
+        <v>0</v>
+      </c>
+      <c r="N108" t="n">
+        <v>0</v>
+      </c>
+      <c r="O108" t="n">
+        <v>0</v>
+      </c>
+      <c r="P108" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q108" t="n">
+        <v>0</v>
+      </c>
+      <c r="R108" t="n">
+        <v>0</v>
+      </c>
+      <c r="S108" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>в том числе: Северная (скандинавская) ходьба</t>
+        </is>
+      </c>
+      <c r="B109" t="n">
+        <v>188</v>
+      </c>
+      <c r="C109" t="n">
+        <v>0</v>
+      </c>
+      <c r="D109" t="n">
+        <v>0</v>
+      </c>
+      <c r="E109" t="n">
+        <v>0</v>
+      </c>
+      <c r="F109" t="n">
+        <v>0</v>
+      </c>
+      <c r="G109" t="n">
+        <v>0</v>
+      </c>
+      <c r="H109" t="n">
+        <v>0</v>
+      </c>
+      <c r="I109" t="n">
+        <v>0</v>
+      </c>
+      <c r="J109" t="n">
+        <v>0</v>
+      </c>
+      <c r="K109" t="n">
+        <v>0</v>
+      </c>
+      <c r="L109" t="n">
+        <v>0</v>
+      </c>
+      <c r="M109" t="n">
+        <v>0</v>
+      </c>
+      <c r="N109" t="n">
+        <v>0</v>
+      </c>
+      <c r="O109" t="n">
+        <v>0</v>
+      </c>
+      <c r="P109" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q109" t="n">
+        <v>0</v>
+      </c>
+      <c r="R109" t="n">
+        <v>0</v>
+      </c>
+      <c r="S109" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Стендовая стрельба</t>
+        </is>
+      </c>
+      <c r="B110" t="n">
+        <v>189</v>
+      </c>
+      <c r="C110" t="n">
+        <v>0</v>
+      </c>
+      <c r="D110" t="n">
+        <v>0</v>
+      </c>
+      <c r="E110" t="n">
+        <v>0</v>
+      </c>
+      <c r="F110" t="n">
+        <v>0</v>
+      </c>
+      <c r="G110" t="n">
+        <v>0</v>
+      </c>
+      <c r="H110" t="n">
+        <v>0</v>
+      </c>
+      <c r="I110" t="n">
+        <v>0</v>
+      </c>
+      <c r="J110" t="n">
+        <v>0</v>
+      </c>
+      <c r="K110" t="n">
+        <v>0</v>
+      </c>
+      <c r="L110" t="n">
+        <v>0</v>
+      </c>
+      <c r="M110" t="n">
+        <v>0</v>
+      </c>
+      <c r="N110" t="n">
+        <v>0</v>
+      </c>
+      <c r="O110" t="n">
+        <v>0</v>
+      </c>
+      <c r="P110" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q110" t="n">
+        <v>0</v>
+      </c>
+      <c r="R110" t="n">
+        <v>0</v>
+      </c>
+      <c r="S110" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Стрельба из арбалета</t>
+        </is>
+      </c>
+      <c r="B111" t="n">
+        <v>190</v>
+      </c>
+      <c r="C111" t="n">
+        <v>0</v>
+      </c>
+      <c r="D111" t="n">
+        <v>0</v>
+      </c>
+      <c r="E111" t="n">
+        <v>0</v>
+      </c>
+      <c r="F111" t="n">
+        <v>0</v>
+      </c>
+      <c r="G111" t="n">
+        <v>0</v>
+      </c>
+      <c r="H111" t="n">
+        <v>0</v>
+      </c>
+      <c r="I111" t="n">
+        <v>0</v>
+      </c>
+      <c r="J111" t="n">
+        <v>0</v>
+      </c>
+      <c r="K111" t="n">
+        <v>0</v>
+      </c>
+      <c r="L111" t="n">
+        <v>0</v>
+      </c>
+      <c r="M111" t="n">
+        <v>0</v>
+      </c>
+      <c r="N111" t="n">
+        <v>0</v>
+      </c>
+      <c r="O111" t="n">
+        <v>0</v>
+      </c>
+      <c r="P111" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q111" t="n">
+        <v>0</v>
+      </c>
+      <c r="R111" t="n">
+        <v>0</v>
+      </c>
+      <c r="S111" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Стрельба из лука</t>
+        </is>
+      </c>
+      <c r="B112" t="n">
+        <v>191</v>
+      </c>
+      <c r="C112" t="n">
+        <v>0</v>
+      </c>
+      <c r="D112" t="n">
+        <v>0</v>
+      </c>
+      <c r="E112" t="n">
+        <v>0</v>
+      </c>
+      <c r="F112" t="n">
+        <v>0</v>
+      </c>
+      <c r="G112" t="n">
+        <v>0</v>
+      </c>
+      <c r="H112" t="n">
+        <v>0</v>
+      </c>
+      <c r="I112" t="n">
+        <v>0</v>
+      </c>
+      <c r="J112" t="n">
+        <v>0</v>
+      </c>
+      <c r="K112" t="n">
+        <v>0</v>
+      </c>
+      <c r="L112" t="n">
+        <v>0</v>
+      </c>
+      <c r="M112" t="n">
+        <v>0</v>
+      </c>
+      <c r="N112" t="n">
+        <v>0</v>
+      </c>
+      <c r="O112" t="n">
+        <v>0</v>
+      </c>
+      <c r="P112" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q112" t="n">
+        <v>0</v>
+      </c>
+      <c r="R112" t="n">
+        <v>0</v>
+      </c>
+      <c r="S112" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Судомодельный спорт</t>
+        </is>
+      </c>
+      <c r="B113" t="n">
+        <v>192</v>
+      </c>
+      <c r="C113" t="n">
+        <v>21</v>
+      </c>
+      <c r="D113" t="n">
+        <v>2</v>
+      </c>
+      <c r="E113" t="n">
+        <v>0</v>
+      </c>
+      <c r="F113" t="n">
+        <v>0</v>
+      </c>
+      <c r="G113" t="n">
+        <v>0</v>
+      </c>
+      <c r="H113" t="n">
+        <v>0</v>
+      </c>
+      <c r="I113" t="n">
+        <v>0</v>
+      </c>
+      <c r="J113" t="n">
+        <v>0</v>
+      </c>
+      <c r="K113" t="n">
+        <v>0</v>
+      </c>
+      <c r="L113" t="n">
+        <v>0</v>
+      </c>
+      <c r="M113" t="n">
+        <v>0</v>
+      </c>
+      <c r="N113" t="n">
+        <v>0</v>
+      </c>
+      <c r="O113" t="n">
+        <v>0</v>
+      </c>
+      <c r="P113" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q113" t="n">
+        <v>0</v>
+      </c>
+      <c r="R113" t="n">
+        <v>0</v>
+      </c>
+      <c r="S113" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>Сумо</t>
+        </is>
+      </c>
+      <c r="B114" t="n">
+        <v>193</v>
+      </c>
+      <c r="C114" t="n">
+        <v>0</v>
+      </c>
+      <c r="D114" t="n">
+        <v>0</v>
+      </c>
+      <c r="E114" t="n">
+        <v>0</v>
+      </c>
+      <c r="F114" t="n">
+        <v>0</v>
+      </c>
+      <c r="G114" t="n">
+        <v>0</v>
+      </c>
+      <c r="H114" t="n">
+        <v>0</v>
+      </c>
+      <c r="I114" t="n">
+        <v>0</v>
+      </c>
+      <c r="J114" t="n">
+        <v>0</v>
+      </c>
+      <c r="K114" t="n">
+        <v>0</v>
+      </c>
+      <c r="L114" t="n">
+        <v>0</v>
+      </c>
+      <c r="M114" t="n">
+        <v>0</v>
+      </c>
+      <c r="N114" t="n">
+        <v>0</v>
+      </c>
+      <c r="O114" t="n">
+        <v>0</v>
+      </c>
+      <c r="P114" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q114" t="n">
+        <v>0</v>
+      </c>
+      <c r="R114" t="n">
+        <v>0</v>
+      </c>
+      <c r="S114" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Тайский бокс</t>
+        </is>
+      </c>
+      <c r="B115" t="n">
+        <v>194</v>
+      </c>
+      <c r="C115" t="n">
+        <v>0</v>
+      </c>
+      <c r="D115" t="n">
+        <v>0</v>
+      </c>
+      <c r="E115" t="n">
+        <v>0</v>
+      </c>
+      <c r="F115" t="n">
+        <v>0</v>
+      </c>
+      <c r="G115" t="n">
+        <v>0</v>
+      </c>
+      <c r="H115" t="n">
+        <v>0</v>
+      </c>
+      <c r="I115" t="n">
+        <v>0</v>
+      </c>
+      <c r="J115" t="n">
+        <v>0</v>
+      </c>
+      <c r="K115" t="n">
+        <v>0</v>
+      </c>
+      <c r="L115" t="n">
+        <v>0</v>
+      </c>
+      <c r="M115" t="n">
+        <v>0</v>
+      </c>
+      <c r="N115" t="n">
+        <v>0</v>
+      </c>
+      <c r="O115" t="n">
+        <v>0</v>
+      </c>
+      <c r="P115" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q115" t="n">
+        <v>0</v>
+      </c>
+      <c r="R115" t="n">
+        <v>0</v>
+      </c>
+      <c r="S115" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>Танцевальный спорт</t>
+        </is>
+      </c>
+      <c r="B116" t="n">
+        <v>195</v>
+      </c>
+      <c r="C116" t="n">
+        <v>0</v>
+      </c>
+      <c r="D116" t="n">
+        <v>0</v>
+      </c>
+      <c r="E116" t="n">
+        <v>0</v>
+      </c>
+      <c r="F116" t="n">
+        <v>0</v>
+      </c>
+      <c r="G116" t="n">
+        <v>0</v>
+      </c>
+      <c r="H116" t="n">
+        <v>0</v>
+      </c>
+      <c r="I116" t="n">
+        <v>0</v>
+      </c>
+      <c r="J116" t="n">
+        <v>0</v>
+      </c>
+      <c r="K116" t="n">
+        <v>0</v>
+      </c>
+      <c r="L116" t="n">
+        <v>0</v>
+      </c>
+      <c r="M116" t="n">
+        <v>0</v>
+      </c>
+      <c r="N116" t="n">
+        <v>0</v>
+      </c>
+      <c r="O116" t="n">
+        <v>0</v>
+      </c>
+      <c r="P116" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q116" t="n">
+        <v>0</v>
+      </c>
+      <c r="R116" t="n">
+        <v>0</v>
+      </c>
+      <c r="S116" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>Теннис</t>
+        </is>
+      </c>
+      <c r="B117" t="n">
+        <v>196</v>
+      </c>
+      <c r="C117" t="n">
+        <v>0</v>
+      </c>
+      <c r="D117" t="n">
+        <v>0</v>
+      </c>
+      <c r="E117" t="n">
+        <v>0</v>
+      </c>
+      <c r="F117" t="n">
+        <v>0</v>
+      </c>
+      <c r="G117" t="n">
+        <v>0</v>
+      </c>
+      <c r="H117" t="n">
+        <v>0</v>
+      </c>
+      <c r="I117" t="n">
+        <v>0</v>
+      </c>
+      <c r="J117" t="n">
+        <v>0</v>
+      </c>
+      <c r="K117" t="n">
+        <v>0</v>
+      </c>
+      <c r="L117" t="n">
+        <v>0</v>
+      </c>
+      <c r="M117" t="n">
+        <v>0</v>
+      </c>
+      <c r="N117" t="n">
+        <v>0</v>
+      </c>
+      <c r="O117" t="n">
+        <v>0</v>
+      </c>
+      <c r="P117" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q117" t="n">
+        <v>0</v>
+      </c>
+      <c r="R117" t="n">
+        <v>0</v>
+      </c>
+      <c r="S117" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>Триатлон</t>
+        </is>
+      </c>
+      <c r="B118" t="n">
+        <v>197</v>
+      </c>
+      <c r="C118" t="n">
+        <v>0</v>
+      </c>
+      <c r="D118" t="n">
+        <v>0</v>
+      </c>
+      <c r="E118" t="n">
+        <v>0</v>
+      </c>
+      <c r="F118" t="n">
+        <v>0</v>
+      </c>
+      <c r="G118" t="n">
+        <v>0</v>
+      </c>
+      <c r="H118" t="n">
+        <v>0</v>
+      </c>
+      <c r="I118" t="n">
+        <v>0</v>
+      </c>
+      <c r="J118" t="n">
+        <v>0</v>
+      </c>
+      <c r="K118" t="n">
+        <v>0</v>
+      </c>
+      <c r="L118" t="n">
+        <v>0</v>
+      </c>
+      <c r="M118" t="n">
+        <v>0</v>
+      </c>
+      <c r="N118" t="n">
+        <v>0</v>
+      </c>
+      <c r="O118" t="n">
+        <v>0</v>
+      </c>
+      <c r="P118" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q118" t="n">
+        <v>0</v>
+      </c>
+      <c r="R118" t="n">
+        <v>0</v>
+      </c>
+      <c r="S118" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>Тхэквондо</t>
+        </is>
+      </c>
+      <c r="B119" t="n">
+        <v>198</v>
+      </c>
+      <c r="C119" t="n">
+        <v>0</v>
+      </c>
+      <c r="D119" t="n">
+        <v>0</v>
+      </c>
+      <c r="E119" t="n">
+        <v>0</v>
+      </c>
+      <c r="F119" t="n">
+        <v>0</v>
+      </c>
+      <c r="G119" t="n">
+        <v>0</v>
+      </c>
+      <c r="H119" t="n">
+        <v>0</v>
+      </c>
+      <c r="I119" t="n">
+        <v>0</v>
+      </c>
+      <c r="J119" t="n">
+        <v>0</v>
+      </c>
+      <c r="K119" t="n">
+        <v>0</v>
+      </c>
+      <c r="L119" t="n">
+        <v>0</v>
+      </c>
+      <c r="M119" t="n">
+        <v>0</v>
+      </c>
+      <c r="N119" t="n">
+        <v>0</v>
+      </c>
+      <c r="O119" t="n">
+        <v>0</v>
+      </c>
+      <c r="P119" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q119" t="n">
+        <v>0</v>
+      </c>
+      <c r="R119" t="n">
+        <v>0</v>
+      </c>
+      <c r="S119" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>Тхэквондо ИТФ</t>
+        </is>
+      </c>
+      <c r="B120" t="n">
+        <v>199</v>
+      </c>
+      <c r="C120" t="n">
+        <v>0</v>
+      </c>
+      <c r="D120" t="n">
+        <v>0</v>
+      </c>
+      <c r="E120" t="n">
+        <v>0</v>
+      </c>
+      <c r="F120" t="n">
+        <v>0</v>
+      </c>
+      <c r="G120" t="n">
+        <v>0</v>
+      </c>
+      <c r="H120" t="n">
+        <v>0</v>
+      </c>
+      <c r="I120" t="n">
+        <v>0</v>
+      </c>
+      <c r="J120" t="n">
+        <v>0</v>
+      </c>
+      <c r="K120" t="n">
+        <v>0</v>
+      </c>
+      <c r="L120" t="n">
+        <v>0</v>
+      </c>
+      <c r="M120" t="n">
+        <v>0</v>
+      </c>
+      <c r="N120" t="n">
+        <v>0</v>
+      </c>
+      <c r="O120" t="n">
+        <v>0</v>
+      </c>
+      <c r="P120" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q120" t="n">
+        <v>0</v>
+      </c>
+      <c r="R120" t="n">
+        <v>0</v>
+      </c>
+      <c r="S120" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>Тяжелая атлетика</t>
+        </is>
+      </c>
+      <c r="B121" t="n">
+        <v>200</v>
+      </c>
+      <c r="C121" t="n">
+        <v>135</v>
+      </c>
+      <c r="D121" t="n">
+        <v>0</v>
+      </c>
+      <c r="E121" t="n">
+        <v>0</v>
+      </c>
+      <c r="F121" t="n">
+        <v>0</v>
+      </c>
+      <c r="G121" t="n">
+        <v>0</v>
+      </c>
+      <c r="H121" t="n">
+        <v>0</v>
+      </c>
+      <c r="I121" t="n">
+        <v>0</v>
+      </c>
+      <c r="J121" t="n">
+        <v>0</v>
+      </c>
+      <c r="K121" t="n">
+        <v>0</v>
+      </c>
+      <c r="L121" t="n">
+        <v>0</v>
+      </c>
+      <c r="M121" t="n">
+        <v>0</v>
+      </c>
+      <c r="N121" t="n">
+        <v>0</v>
+      </c>
+      <c r="O121" t="n">
+        <v>0</v>
+      </c>
+      <c r="P121" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q121" t="n">
+        <v>0</v>
+      </c>
+      <c r="R121" t="n">
+        <v>0</v>
+      </c>
+      <c r="S121" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>Универсальный бой</t>
+        </is>
+      </c>
+      <c r="B122" t="n">
+        <v>201</v>
+      </c>
+      <c r="C122" t="n">
+        <v>216</v>
+      </c>
+      <c r="D122" t="n">
+        <v>0</v>
+      </c>
+      <c r="E122" t="n">
+        <v>0</v>
+      </c>
+      <c r="F122" t="n">
+        <v>0</v>
+      </c>
+      <c r="G122" t="n">
+        <v>0</v>
+      </c>
+      <c r="H122" t="n">
+        <v>0</v>
+      </c>
+      <c r="I122" t="n">
+        <v>0</v>
+      </c>
+      <c r="J122" t="n">
+        <v>0</v>
+      </c>
+      <c r="K122" t="n">
+        <v>0</v>
+      </c>
+      <c r="L122" t="n">
+        <v>0</v>
+      </c>
+      <c r="M122" t="n">
+        <v>0</v>
+      </c>
+      <c r="N122" t="n">
+        <v>0</v>
+      </c>
+      <c r="O122" t="n">
+        <v>0</v>
+      </c>
+      <c r="P122" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q122" t="n">
+        <v>0</v>
+      </c>
+      <c r="R122" t="n">
+        <v>0</v>
+      </c>
+      <c r="S122" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>Ушу</t>
+        </is>
+      </c>
+      <c r="B123" t="n">
+        <v>202</v>
+      </c>
+      <c r="C123" t="n">
+        <v>0</v>
+      </c>
+      <c r="D123" t="n">
+        <v>0</v>
+      </c>
+      <c r="E123" t="n">
+        <v>0</v>
+      </c>
+      <c r="F123" t="n">
+        <v>0</v>
+      </c>
+      <c r="G123" t="n">
+        <v>0</v>
+      </c>
+      <c r="H123" t="n">
+        <v>0</v>
+      </c>
+      <c r="I123" t="n">
+        <v>0</v>
+      </c>
+      <c r="J123" t="n">
+        <v>0</v>
+      </c>
+      <c r="K123" t="n">
+        <v>0</v>
+      </c>
+      <c r="L123" t="n">
+        <v>0</v>
+      </c>
+      <c r="M123" t="n">
+        <v>0</v>
+      </c>
+      <c r="N123" t="n">
+        <v>0</v>
+      </c>
+      <c r="O123" t="n">
+        <v>0</v>
+      </c>
+      <c r="P123" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q123" t="n">
+        <v>0</v>
+      </c>
+      <c r="R123" t="n">
+        <v>0</v>
+      </c>
+      <c r="S123" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>Фехтование</t>
+        </is>
+      </c>
+      <c r="B124" t="n">
+        <v>203</v>
+      </c>
+      <c r="C124" t="n">
+        <v>0</v>
+      </c>
+      <c r="D124" t="n">
+        <v>0</v>
+      </c>
+      <c r="E124" t="n">
+        <v>0</v>
+      </c>
+      <c r="F124" t="n">
+        <v>0</v>
+      </c>
+      <c r="G124" t="n">
+        <v>0</v>
+      </c>
+      <c r="H124" t="n">
+        <v>0</v>
+      </c>
+      <c r="I124" t="n">
+        <v>0</v>
+      </c>
+      <c r="J124" t="n">
+        <v>0</v>
+      </c>
+      <c r="K124" t="n">
+        <v>0</v>
+      </c>
+      <c r="L124" t="n">
+        <v>0</v>
+      </c>
+      <c r="M124" t="n">
+        <v>0</v>
+      </c>
+      <c r="N124" t="n">
+        <v>0</v>
+      </c>
+      <c r="O124" t="n">
+        <v>0</v>
+      </c>
+      <c r="P124" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q124" t="n">
+        <v>0</v>
+      </c>
+      <c r="R124" t="n">
+        <v>0</v>
+      </c>
+      <c r="S124" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>Фигурное катание на коньках</t>
+        </is>
+      </c>
+      <c r="B125" t="n">
+        <v>204</v>
+      </c>
+      <c r="C125" t="n">
+        <v>0</v>
+      </c>
+      <c r="D125" t="n">
+        <v>0</v>
+      </c>
+      <c r="E125" t="n">
+        <v>0</v>
+      </c>
+      <c r="F125" t="n">
+        <v>0</v>
+      </c>
+      <c r="G125" t="n">
+        <v>0</v>
+      </c>
+      <c r="H125" t="n">
+        <v>0</v>
+      </c>
+      <c r="I125" t="n">
+        <v>0</v>
+      </c>
+      <c r="J125" t="n">
+        <v>0</v>
+      </c>
+      <c r="K125" t="n">
+        <v>0</v>
+      </c>
+      <c r="L125" t="n">
+        <v>0</v>
+      </c>
+      <c r="M125" t="n">
+        <v>0</v>
+      </c>
+      <c r="N125" t="n">
+        <v>0</v>
+      </c>
+      <c r="O125" t="n">
+        <v>0</v>
+      </c>
+      <c r="P125" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q125" t="n">
+        <v>0</v>
+      </c>
+      <c r="R125" t="n">
+        <v>0</v>
+      </c>
+      <c r="S125" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>Фитнес-аэробика</t>
+        </is>
+      </c>
+      <c r="B126" t="n">
+        <v>205</v>
+      </c>
+      <c r="C126" t="n">
+        <v>25</v>
+      </c>
+      <c r="D126" t="n">
+        <v>20</v>
+      </c>
+      <c r="E126" t="n">
+        <v>0</v>
+      </c>
+      <c r="F126" t="n">
+        <v>0</v>
+      </c>
+      <c r="G126" t="n">
+        <v>0</v>
+      </c>
+      <c r="H126" t="n">
+        <v>0</v>
+      </c>
+      <c r="I126" t="n">
+        <v>0</v>
+      </c>
+      <c r="J126" t="n">
+        <v>0</v>
+      </c>
+      <c r="K126" t="n">
+        <v>0</v>
+      </c>
+      <c r="L126" t="n">
+        <v>0</v>
+      </c>
+      <c r="M126" t="n">
+        <v>0</v>
+      </c>
+      <c r="N126" t="n">
+        <v>0</v>
+      </c>
+      <c r="O126" t="n">
+        <v>0</v>
+      </c>
+      <c r="P126" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q126" t="n">
+        <v>0</v>
+      </c>
+      <c r="R126" t="n">
+        <v>0</v>
+      </c>
+      <c r="S126" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>Флорбол</t>
+        </is>
+      </c>
+      <c r="B127" t="n">
+        <v>206</v>
+      </c>
+      <c r="C127" t="n">
+        <v>0</v>
+      </c>
+      <c r="D127" t="n">
+        <v>0</v>
+      </c>
+      <c r="E127" t="n">
+        <v>0</v>
+      </c>
+      <c r="F127" t="n">
+        <v>0</v>
+      </c>
+      <c r="G127" t="n">
+        <v>0</v>
+      </c>
+      <c r="H127" t="n">
+        <v>0</v>
+      </c>
+      <c r="I127" t="n">
+        <v>0</v>
+      </c>
+      <c r="J127" t="n">
+        <v>0</v>
+      </c>
+      <c r="K127" t="n">
+        <v>0</v>
+      </c>
+      <c r="L127" t="n">
+        <v>0</v>
+      </c>
+      <c r="M127" t="n">
+        <v>0</v>
+      </c>
+      <c r="N127" t="n">
+        <v>0</v>
+      </c>
+      <c r="O127" t="n">
+        <v>0</v>
+      </c>
+      <c r="P127" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q127" t="n">
+        <v>0</v>
+      </c>
+      <c r="R127" t="n">
+        <v>0</v>
+      </c>
+      <c r="S127" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>Фристайл</t>
+        </is>
+      </c>
+      <c r="B128" t="n">
+        <v>207</v>
+      </c>
+      <c r="C128" t="n">
+        <v>0</v>
+      </c>
+      <c r="D128" t="n">
+        <v>0</v>
+      </c>
+      <c r="E128" t="n">
+        <v>0</v>
+      </c>
+      <c r="F128" t="n">
+        <v>0</v>
+      </c>
+      <c r="G128" t="n">
+        <v>0</v>
+      </c>
+      <c r="H128" t="n">
+        <v>0</v>
+      </c>
+      <c r="I128" t="n">
+        <v>0</v>
+      </c>
+      <c r="J128" t="n">
+        <v>0</v>
+      </c>
+      <c r="K128" t="n">
+        <v>0</v>
+      </c>
+      <c r="L128" t="n">
+        <v>0</v>
+      </c>
+      <c r="M128" t="n">
+        <v>0</v>
+      </c>
+      <c r="N128" t="n">
+        <v>0</v>
+      </c>
+      <c r="O128" t="n">
+        <v>0</v>
+      </c>
+      <c r="P128" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q128" t="n">
+        <v>0</v>
+      </c>
+      <c r="R128" t="n">
+        <v>0</v>
+      </c>
+      <c r="S128" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>Функциональное многоборье</t>
+        </is>
+      </c>
+      <c r="B129" t="n">
+        <v>208</v>
+      </c>
+      <c r="C129" t="n">
+        <v>0</v>
+      </c>
+      <c r="D129" t="n">
+        <v>0</v>
+      </c>
+      <c r="E129" t="n">
+        <v>0</v>
+      </c>
+      <c r="F129" t="n">
+        <v>0</v>
+      </c>
+      <c r="G129" t="n">
+        <v>0</v>
+      </c>
+      <c r="H129" t="n">
+        <v>0</v>
+      </c>
+      <c r="I129" t="n">
+        <v>0</v>
+      </c>
+      <c r="J129" t="n">
+        <v>0</v>
+      </c>
+      <c r="K129" t="n">
+        <v>0</v>
+      </c>
+      <c r="L129" t="n">
+        <v>0</v>
+      </c>
+      <c r="M129" t="n">
+        <v>0</v>
+      </c>
+      <c r="N129" t="n">
+        <v>0</v>
+      </c>
+      <c r="O129" t="n">
+        <v>0</v>
+      </c>
+      <c r="P129" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q129" t="n">
+        <v>0</v>
+      </c>
+      <c r="R129" t="n">
+        <v>0</v>
+      </c>
+      <c r="S129" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>Футбол</t>
+        </is>
+      </c>
+      <c r="B130" t="n">
+        <v>209</v>
+      </c>
+      <c r="C130" t="n">
+        <v>488</v>
+      </c>
+      <c r="D130" t="n">
+        <v>42</v>
+      </c>
+      <c r="E130" t="n">
+        <v>0</v>
+      </c>
+      <c r="F130" t="n">
+        <v>0</v>
+      </c>
+      <c r="G130" t="n">
+        <v>0</v>
+      </c>
+      <c r="H130" t="n">
+        <v>0</v>
+      </c>
+      <c r="I130" t="n">
+        <v>0</v>
+      </c>
+      <c r="J130" t="n">
+        <v>0</v>
+      </c>
+      <c r="K130" t="n">
+        <v>0</v>
+      </c>
+      <c r="L130" t="n">
+        <v>1</v>
+      </c>
+      <c r="M130" t="n">
+        <v>0</v>
+      </c>
+      <c r="N130" t="n">
+        <v>0</v>
+      </c>
+      <c r="O130" t="n">
+        <v>7</v>
+      </c>
+      <c r="P130" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q130" t="n">
+        <v>6</v>
+      </c>
+      <c r="R130" t="n">
+        <v>0</v>
+      </c>
+      <c r="S130" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>Хоккей</t>
+        </is>
+      </c>
+      <c r="B131" t="n">
+        <v>210</v>
+      </c>
+      <c r="C131" t="n">
+        <v>108</v>
+      </c>
+      <c r="D131" t="n">
+        <v>8</v>
+      </c>
+      <c r="E131" t="n">
+        <v>0</v>
+      </c>
+      <c r="F131" t="n">
+        <v>0</v>
+      </c>
+      <c r="G131" t="n">
+        <v>0</v>
+      </c>
+      <c r="H131" t="n">
+        <v>0</v>
+      </c>
+      <c r="I131" t="n">
+        <v>0</v>
+      </c>
+      <c r="J131" t="n">
+        <v>0</v>
+      </c>
+      <c r="K131" t="n">
+        <v>0</v>
+      </c>
+      <c r="L131" t="n">
+        <v>0</v>
+      </c>
+      <c r="M131" t="n">
+        <v>0</v>
+      </c>
+      <c r="N131" t="n">
+        <v>0</v>
+      </c>
+      <c r="O131" t="n">
+        <v>2</v>
+      </c>
+      <c r="P131" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q131" t="n">
+        <v>1</v>
+      </c>
+      <c r="R131" t="n">
+        <v>0</v>
+      </c>
+      <c r="S131" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>Хоккей на траве</t>
+        </is>
+      </c>
+      <c r="B132" t="n">
+        <v>211</v>
+      </c>
+      <c r="C132" t="n">
+        <v>0</v>
+      </c>
+      <c r="D132" t="n">
+        <v>0</v>
+      </c>
+      <c r="E132" t="n">
+        <v>0</v>
+      </c>
+      <c r="F132" t="n">
+        <v>0</v>
+      </c>
+      <c r="G132" t="n">
+        <v>0</v>
+      </c>
+      <c r="H132" t="n">
+        <v>0</v>
+      </c>
+      <c r="I132" t="n">
+        <v>0</v>
+      </c>
+      <c r="J132" t="n">
+        <v>0</v>
+      </c>
+      <c r="K132" t="n">
+        <v>0</v>
+      </c>
+      <c r="L132" t="n">
+        <v>0</v>
+      </c>
+      <c r="M132" t="n">
+        <v>0</v>
+      </c>
+      <c r="N132" t="n">
+        <v>0</v>
+      </c>
+      <c r="O132" t="n">
+        <v>0</v>
+      </c>
+      <c r="P132" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q132" t="n">
+        <v>0</v>
+      </c>
+      <c r="R132" t="n">
+        <v>0</v>
+      </c>
+      <c r="S132" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>Хоккей с мячом</t>
+        </is>
+      </c>
+      <c r="B133" t="n">
+        <v>212</v>
+      </c>
+      <c r="C133" t="n">
+        <v>0</v>
+      </c>
+      <c r="D133" t="n">
+        <v>0</v>
+      </c>
+      <c r="E133" t="n">
+        <v>0</v>
+      </c>
+      <c r="F133" t="n">
+        <v>0</v>
+      </c>
+      <c r="G133" t="n">
+        <v>0</v>
+      </c>
+      <c r="H133" t="n">
+        <v>0</v>
+      </c>
+      <c r="I133" t="n">
+        <v>0</v>
+      </c>
+      <c r="J133" t="n">
+        <v>0</v>
+      </c>
+      <c r="K133" t="n">
+        <v>0</v>
+      </c>
+      <c r="L133" t="n">
+        <v>0</v>
+      </c>
+      <c r="M133" t="n">
+        <v>0</v>
+      </c>
+      <c r="N133" t="n">
+        <v>0</v>
+      </c>
+      <c r="O133" t="n">
+        <v>0</v>
+      </c>
+      <c r="P133" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q133" t="n">
+        <v>0</v>
+      </c>
+      <c r="R133" t="n">
+        <v>0</v>
+      </c>
+      <c r="S133" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>Художественная гимнастика</t>
+        </is>
+      </c>
+      <c r="B134" t="n">
+        <v>213</v>
+      </c>
+      <c r="C134" t="n">
+        <v>0</v>
+      </c>
+      <c r="D134" t="n">
+        <v>0</v>
+      </c>
+      <c r="E134" t="n">
+        <v>0</v>
+      </c>
+      <c r="F134" t="n">
+        <v>0</v>
+      </c>
+      <c r="G134" t="n">
+        <v>0</v>
+      </c>
+      <c r="H134" t="n">
+        <v>0</v>
+      </c>
+      <c r="I134" t="n">
+        <v>0</v>
+      </c>
+      <c r="J134" t="n">
+        <v>0</v>
+      </c>
+      <c r="K134" t="n">
+        <v>0</v>
+      </c>
+      <c r="L134" t="n">
+        <v>0</v>
+      </c>
+      <c r="M134" t="n">
+        <v>0</v>
+      </c>
+      <c r="N134" t="n">
+        <v>0</v>
+      </c>
+      <c r="O134" t="n">
+        <v>0</v>
+      </c>
+      <c r="P134" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q134" t="n">
+        <v>0</v>
+      </c>
+      <c r="R134" t="n">
+        <v>0</v>
+      </c>
+      <c r="S134" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>Чир спорт</t>
+        </is>
+      </c>
+      <c r="B135" t="n">
+        <v>214</v>
+      </c>
+      <c r="C135" t="n">
+        <v>0</v>
+      </c>
+      <c r="D135" t="n">
+        <v>0</v>
+      </c>
+      <c r="E135" t="n">
+        <v>0</v>
+      </c>
+      <c r="F135" t="n">
+        <v>0</v>
+      </c>
+      <c r="G135" t="n">
+        <v>0</v>
+      </c>
+      <c r="H135" t="n">
+        <v>0</v>
+      </c>
+      <c r="I135" t="n">
+        <v>0</v>
+      </c>
+      <c r="J135" t="n">
+        <v>0</v>
+      </c>
+      <c r="K135" t="n">
+        <v>0</v>
+      </c>
+      <c r="L135" t="n">
+        <v>0</v>
+      </c>
+      <c r="M135" t="n">
+        <v>0</v>
+      </c>
+      <c r="N135" t="n">
+        <v>0</v>
+      </c>
+      <c r="O135" t="n">
+        <v>0</v>
+      </c>
+      <c r="P135" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q135" t="n">
+        <v>0</v>
+      </c>
+      <c r="R135" t="n">
+        <v>0</v>
+      </c>
+      <c r="S135" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>Шахматы</t>
+        </is>
+      </c>
+      <c r="B136" t="n">
+        <v>215</v>
+      </c>
+      <c r="C136" t="n">
+        <v>145</v>
+      </c>
+      <c r="D136" t="n">
+        <v>30</v>
+      </c>
+      <c r="E136" t="n">
+        <v>0</v>
+      </c>
+      <c r="F136" t="n">
+        <v>0</v>
+      </c>
+      <c r="G136" t="n">
+        <v>0</v>
+      </c>
+      <c r="H136" t="n">
+        <v>0</v>
+      </c>
+      <c r="I136" t="n">
+        <v>0</v>
+      </c>
+      <c r="J136" t="n">
+        <v>0</v>
+      </c>
+      <c r="K136" t="n">
+        <v>0</v>
+      </c>
+      <c r="L136" t="n">
+        <v>1</v>
+      </c>
+      <c r="M136" t="n">
+        <v>1</v>
+      </c>
+      <c r="N136" t="n">
+        <v>0</v>
+      </c>
+      <c r="O136" t="n">
+        <v>3</v>
+      </c>
+      <c r="P136" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q136" t="n">
+        <v>1</v>
+      </c>
+      <c r="R136" t="n">
+        <v>0</v>
+      </c>
+      <c r="S136" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>Шашки</t>
+        </is>
+      </c>
+      <c r="B137" t="n">
+        <v>216</v>
+      </c>
+      <c r="C137" t="n">
+        <v>49</v>
+      </c>
+      <c r="D137" t="n">
+        <v>34</v>
+      </c>
+      <c r="E137" t="n">
+        <v>0</v>
+      </c>
+      <c r="F137" t="n">
+        <v>0</v>
+      </c>
+      <c r="G137" t="n">
+        <v>0</v>
+      </c>
+      <c r="H137" t="n">
+        <v>0</v>
+      </c>
+      <c r="I137" t="n">
+        <v>0</v>
+      </c>
+      <c r="J137" t="n">
+        <v>0</v>
+      </c>
+      <c r="K137" t="n">
+        <v>0</v>
+      </c>
+      <c r="L137" t="n">
+        <v>0</v>
+      </c>
+      <c r="M137" t="n">
+        <v>0</v>
+      </c>
+      <c r="N137" t="n">
+        <v>0</v>
+      </c>
+      <c r="O137" t="n">
+        <v>0</v>
+      </c>
+      <c r="P137" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q137" t="n">
+        <v>0</v>
+      </c>
+      <c r="R137" t="n">
+        <v>0</v>
+      </c>
+      <c r="S137" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>Эстетическая гимнастика</t>
+        </is>
+      </c>
+      <c r="B138" t="n">
+        <v>217</v>
+      </c>
+      <c r="C138" t="n">
+        <v>25</v>
+      </c>
+      <c r="D138" t="n">
+        <v>16</v>
+      </c>
+      <c r="E138" t="n">
+        <v>0</v>
+      </c>
+      <c r="F138" t="n">
+        <v>0</v>
+      </c>
+      <c r="G138" t="n">
+        <v>0</v>
+      </c>
+      <c r="H138" t="n">
+        <v>0</v>
+      </c>
+      <c r="I138" t="n">
+        <v>0</v>
+      </c>
+      <c r="J138" t="n">
+        <v>0</v>
+      </c>
+      <c r="K138" t="n">
+        <v>0</v>
+      </c>
+      <c r="L138" t="n">
+        <v>0</v>
+      </c>
+      <c r="M138" t="n">
+        <v>0</v>
+      </c>
+      <c r="N138" t="n">
+        <v>0</v>
+      </c>
+      <c r="O138" t="n">
+        <v>0</v>
+      </c>
+      <c r="P138" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q138" t="n">
+        <v>0</v>
+      </c>
+      <c r="R138" t="n">
+        <v>0</v>
+      </c>
+      <c r="S138" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>Прикладные виды спорта – всего(сумма строк 219-220)</t>
+        </is>
+      </c>
+      <c r="B139" t="n">
+        <v>218</v>
+      </c>
+      <c r="C139" t="n">
+        <v>35</v>
+      </c>
+      <c r="D139" t="n">
+        <v>14</v>
+      </c>
+      <c r="E139" t="n">
+        <v>0</v>
+      </c>
+      <c r="F139" t="n">
+        <v>0</v>
+      </c>
+      <c r="G139" t="n">
+        <v>0</v>
+      </c>
+      <c r="H139" t="n">
+        <v>0</v>
+      </c>
+      <c r="I139" t="n">
+        <v>0</v>
+      </c>
+      <c r="J139" t="n">
+        <v>0</v>
+      </c>
+      <c r="K139" t="n">
+        <v>0</v>
+      </c>
+      <c r="L139" t="n">
+        <v>0</v>
+      </c>
+      <c r="M139" t="n">
+        <v>0</v>
+      </c>
+      <c r="N139" t="n">
+        <v>0</v>
+      </c>
+      <c r="O139" t="n">
+        <v>1</v>
+      </c>
+      <c r="P139" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q139" t="n">
+        <v>0</v>
+      </c>
+      <c r="R139" t="n">
+        <v>0</v>
+      </c>
+      <c r="S139" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>в том числе: военно-прикладные</t>
+        </is>
+      </c>
+      <c r="B140" t="n">
+        <v>219</v>
+      </c>
+      <c r="C140" t="n">
+        <v>35</v>
+      </c>
+      <c r="D140" t="n">
+        <v>14</v>
+      </c>
+      <c r="E140" t="n">
+        <v>0</v>
+      </c>
+      <c r="F140" t="n">
+        <v>0</v>
+      </c>
+      <c r="G140" t="n">
+        <v>0</v>
+      </c>
+      <c r="H140" t="n">
+        <v>0</v>
+      </c>
+      <c r="I140" t="n">
+        <v>0</v>
+      </c>
+      <c r="J140" t="n">
+        <v>0</v>
+      </c>
+      <c r="K140" t="n">
+        <v>0</v>
+      </c>
+      <c r="L140" t="n">
+        <v>0</v>
+      </c>
+      <c r="M140" t="n">
+        <v>0</v>
+      </c>
+      <c r="N140" t="n">
+        <v>0</v>
+      </c>
+      <c r="O140" t="n">
+        <v>1</v>
+      </c>
+      <c r="P140" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q140" t="n">
+        <v>0</v>
+      </c>
+      <c r="R140" t="n">
+        <v>0</v>
+      </c>
+      <c r="S140" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>служебно-прикладные</t>
+        </is>
+      </c>
+      <c r="B141" t="n">
+        <v>220</v>
+      </c>
+      <c r="C141" t="n">
+        <v>0</v>
+      </c>
+      <c r="D141" t="n">
+        <v>0</v>
+      </c>
+      <c r="E141" t="n">
+        <v>0</v>
+      </c>
+      <c r="F141" t="n">
+        <v>0</v>
+      </c>
+      <c r="G141" t="n">
+        <v>0</v>
+      </c>
+      <c r="H141" t="n">
+        <v>0</v>
+      </c>
+      <c r="I141" t="n">
+        <v>0</v>
+      </c>
+      <c r="J141" t="n">
+        <v>0</v>
+      </c>
+      <c r="K141" t="n">
+        <v>0</v>
+      </c>
+      <c r="L141" t="n">
+        <v>0</v>
+      </c>
+      <c r="M141" t="n">
+        <v>0</v>
+      </c>
+      <c r="N141" t="n">
+        <v>0</v>
+      </c>
+      <c r="O141" t="n">
+        <v>0</v>
+      </c>
+      <c r="P141" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q141" t="n">
+        <v>0</v>
+      </c>
+      <c r="R141" t="n">
+        <v>0</v>
+      </c>
+      <c r="S141" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>Национальные виды спорта – всего (сумма строк 222-229)</t>
+        </is>
+      </c>
+      <c r="B142" t="n">
+        <v>221</v>
+      </c>
+      <c r="C142" t="n">
+        <v>0</v>
+      </c>
+      <c r="D142" t="n">
+        <v>0</v>
+      </c>
+      <c r="E142" t="n">
+        <v>0</v>
+      </c>
+      <c r="F142" t="n">
+        <v>0</v>
+      </c>
+      <c r="G142" t="n">
+        <v>0</v>
+      </c>
+      <c r="H142" t="n">
+        <v>0</v>
+      </c>
+      <c r="I142" t="n">
+        <v>0</v>
+      </c>
+      <c r="J142" t="n">
+        <v>0</v>
+      </c>
+      <c r="K142" t="n">
+        <v>0</v>
+      </c>
+      <c r="L142" t="n">
+        <v>0</v>
+      </c>
+      <c r="M142" t="n">
+        <v>0</v>
+      </c>
+      <c r="N142" t="n">
+        <v>0</v>
+      </c>
+      <c r="O142" t="n">
+        <v>0</v>
+      </c>
+      <c r="P142" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q142" t="n">
+        <v>0</v>
+      </c>
+      <c r="R142" t="n">
+        <v>0</v>
+      </c>
+      <c r="S142" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>в том числе:гонки на охотничьих лыжах</t>
+        </is>
+      </c>
+      <c r="B143" t="n">
+        <v>222</v>
+      </c>
+      <c r="C143" t="n">
+        <v>0</v>
+      </c>
+      <c r="D143" t="n">
+        <v>0</v>
+      </c>
+      <c r="E143" t="n">
+        <v>0</v>
+      </c>
+      <c r="F143" t="n">
+        <v>0</v>
+      </c>
+      <c r="G143" t="n">
+        <v>0</v>
+      </c>
+      <c r="H143" t="n">
+        <v>0</v>
+      </c>
+      <c r="I143" t="n">
+        <v>0</v>
+      </c>
+      <c r="J143" t="n">
+        <v>0</v>
+      </c>
+      <c r="K143" t="n">
+        <v>0</v>
+      </c>
+      <c r="L143" t="n">
+        <v>0</v>
+      </c>
+      <c r="M143" t="n">
+        <v>0</v>
+      </c>
+      <c r="N143" t="n">
+        <v>0</v>
+      </c>
+      <c r="O143" t="n">
+        <v>0</v>
+      </c>
+      <c r="P143" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q143" t="n">
+        <v>0</v>
+      </c>
+      <c r="R143" t="n">
+        <v>0</v>
+      </c>
+      <c r="S143" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>керешу</t>
+        </is>
+      </c>
+      <c r="B144" t="n">
+        <v>223</v>
+      </c>
+      <c r="C144" t="n">
+        <v>0</v>
+      </c>
+      <c r="D144" t="n">
+        <v>0</v>
+      </c>
+      <c r="E144" t="n">
+        <v>0</v>
+      </c>
+      <c r="F144" t="n">
+        <v>0</v>
+      </c>
+      <c r="G144" t="n">
+        <v>0</v>
+      </c>
+      <c r="H144" t="n">
+        <v>0</v>
+      </c>
+      <c r="I144" t="n">
+        <v>0</v>
+      </c>
+      <c r="J144" t="n">
+        <v>0</v>
+      </c>
+      <c r="K144" t="n">
+        <v>0</v>
+      </c>
+      <c r="L144" t="n">
+        <v>0</v>
+      </c>
+      <c r="M144" t="n">
+        <v>0</v>
+      </c>
+      <c r="N144" t="n">
+        <v>0</v>
+      </c>
+      <c r="O144" t="n">
+        <v>0</v>
+      </c>
+      <c r="P144" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q144" t="n">
+        <v>0</v>
+      </c>
+      <c r="R144" t="n">
+        <v>0</v>
+      </c>
+      <c r="S144" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>мас-рестлинг</t>
+        </is>
+      </c>
+      <c r="B145" t="n">
+        <v>224</v>
+      </c>
+      <c r="C145" t="n">
+        <v>0</v>
+      </c>
+      <c r="D145" t="n">
+        <v>0</v>
+      </c>
+      <c r="E145" t="n">
+        <v>0</v>
+      </c>
+      <c r="F145" t="n">
+        <v>0</v>
+      </c>
+      <c r="G145" t="n">
+        <v>0</v>
+      </c>
+      <c r="H145" t="n">
+        <v>0</v>
+      </c>
+      <c r="I145" t="n">
+        <v>0</v>
+      </c>
+      <c r="J145" t="n">
+        <v>0</v>
+      </c>
+      <c r="K145" t="n">
+        <v>0</v>
+      </c>
+      <c r="L145" t="n">
+        <v>0</v>
+      </c>
+      <c r="M145" t="n">
+        <v>0</v>
+      </c>
+      <c r="N145" t="n">
+        <v>0</v>
+      </c>
+      <c r="O145" t="n">
+        <v>0</v>
+      </c>
+      <c r="P145" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q145" t="n">
+        <v>0</v>
+      </c>
+      <c r="R145" t="n">
+        <v>0</v>
+      </c>
+      <c r="S145" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>таврели</t>
+        </is>
+      </c>
+      <c r="B146" t="n">
+        <v>225</v>
+      </c>
+      <c r="C146" t="n">
+        <v>0</v>
+      </c>
+      <c r="D146" t="n">
+        <v>0</v>
+      </c>
+      <c r="E146" t="n">
+        <v>0</v>
+      </c>
+      <c r="F146" t="n">
+        <v>0</v>
+      </c>
+      <c r="G146" t="n">
+        <v>0</v>
+      </c>
+      <c r="H146" t="n">
+        <v>0</v>
+      </c>
+      <c r="I146" t="n">
+        <v>0</v>
+      </c>
+      <c r="J146" t="n">
+        <v>0</v>
+      </c>
+      <c r="K146" t="n">
+        <v>0</v>
+      </c>
+      <c r="L146" t="n">
+        <v>0</v>
+      </c>
+      <c r="M146" t="n">
+        <v>0</v>
+      </c>
+      <c r="N146" t="n">
+        <v>0</v>
+      </c>
+      <c r="O146" t="n">
+        <v>0</v>
+      </c>
+      <c r="P146" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q146" t="n">
+        <v>0</v>
+      </c>
+      <c r="R146" t="n">
+        <v>0</v>
+      </c>
+      <c r="S146" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>хапсагай</t>
+        </is>
+      </c>
+      <c r="B147" t="n">
+        <v>226</v>
+      </c>
+      <c r="C147" t="n">
+        <v>0</v>
+      </c>
+      <c r="D147" t="n">
+        <v>0</v>
+      </c>
+      <c r="E147" t="n">
+        <v>0</v>
+      </c>
+      <c r="F147" t="n">
+        <v>0</v>
+      </c>
+      <c r="G147" t="n">
+        <v>0</v>
+      </c>
+      <c r="H147" t="n">
+        <v>0</v>
+      </c>
+      <c r="I147" t="n">
+        <v>0</v>
+      </c>
+      <c r="J147" t="n">
+        <v>0</v>
+      </c>
+      <c r="K147" t="n">
+        <v>0</v>
+      </c>
+      <c r="L147" t="n">
+        <v>0</v>
+      </c>
+      <c r="M147" t="n">
+        <v>0</v>
+      </c>
+      <c r="N147" t="n">
+        <v>0</v>
+      </c>
+      <c r="O147" t="n">
+        <v>0</v>
+      </c>
+      <c r="P147" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q147" t="n">
+        <v>0</v>
+      </c>
+      <c r="R147" t="n">
+        <v>0</v>
+      </c>
+      <c r="S147" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>хуреш</t>
+        </is>
+      </c>
+      <c r="B148" t="n">
+        <v>227</v>
+      </c>
+      <c r="C148" t="n">
+        <v>0</v>
+      </c>
+      <c r="D148" t="n">
+        <v>0</v>
+      </c>
+      <c r="E148" t="n">
+        <v>0</v>
+      </c>
+      <c r="F148" t="n">
+        <v>0</v>
+      </c>
+      <c r="G148" t="n">
+        <v>0</v>
+      </c>
+      <c r="H148" t="n">
+        <v>0</v>
+      </c>
+      <c r="I148" t="n">
+        <v>0</v>
+      </c>
+      <c r="J148" t="n">
+        <v>0</v>
+      </c>
+      <c r="K148" t="n">
+        <v>0</v>
+      </c>
+      <c r="L148" t="n">
+        <v>0</v>
+      </c>
+      <c r="M148" t="n">
+        <v>0</v>
+      </c>
+      <c r="N148" t="n">
+        <v>0</v>
+      </c>
+      <c r="O148" t="n">
+        <v>0</v>
+      </c>
+      <c r="P148" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q148" t="n">
+        <v>0</v>
+      </c>
+      <c r="R148" t="n">
+        <v>0</v>
+      </c>
+      <c r="S148" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>шодсанлат</t>
+        </is>
+      </c>
+      <c r="B149" t="n">
+        <v>228</v>
+      </c>
+      <c r="C149" t="n">
+        <v>0</v>
+      </c>
+      <c r="D149" t="n">
+        <v>0</v>
+      </c>
+      <c r="E149" t="n">
+        <v>0</v>
+      </c>
+      <c r="F149" t="n">
+        <v>0</v>
+      </c>
+      <c r="G149" t="n">
+        <v>0</v>
+      </c>
+      <c r="H149" t="n">
+        <v>0</v>
+      </c>
+      <c r="I149" t="n">
+        <v>0</v>
+      </c>
+      <c r="J149" t="n">
+        <v>0</v>
+      </c>
+      <c r="K149" t="n">
+        <v>0</v>
+      </c>
+      <c r="L149" t="n">
+        <v>0</v>
+      </c>
+      <c r="M149" t="n">
+        <v>0</v>
+      </c>
+      <c r="N149" t="n">
+        <v>0</v>
+      </c>
+      <c r="O149" t="n">
+        <v>0</v>
+      </c>
+      <c r="P149" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q149" t="n">
+        <v>0</v>
+      </c>
+      <c r="R149" t="n">
+        <v>0</v>
+      </c>
+      <c r="S149" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>якутские национальные прыжки</t>
+        </is>
+      </c>
+      <c r="B150" t="n">
+        <v>229</v>
+      </c>
+      <c r="C150" t="n">
+        <v>0</v>
+      </c>
+      <c r="D150" t="n">
+        <v>0</v>
+      </c>
+      <c r="E150" t="n">
+        <v>0</v>
+      </c>
+      <c r="F150" t="n">
+        <v>0</v>
+      </c>
+      <c r="G150" t="n">
+        <v>0</v>
+      </c>
+      <c r="H150" t="n">
+        <v>0</v>
+      </c>
+      <c r="I150" t="n">
+        <v>0</v>
+      </c>
+      <c r="J150" t="n">
+        <v>0</v>
+      </c>
+      <c r="K150" t="n">
+        <v>0</v>
+      </c>
+      <c r="L150" t="n">
+        <v>0</v>
+      </c>
+      <c r="M150" t="n">
+        <v>0</v>
+      </c>
+      <c r="N150" t="n">
+        <v>0</v>
+      </c>
+      <c r="O150" t="n">
+        <v>0</v>
+      </c>
+      <c r="P150" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q150" t="n">
+        <v>0</v>
+      </c>
+      <c r="R150" t="n">
+        <v>0</v>
+      </c>
+      <c r="S150" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>Виды спорта, признанные в Российской Федерации (сумма строк 231-240)</t>
+        </is>
+      </c>
+      <c r="B151" t="n">
+        <v>230</v>
+      </c>
+      <c r="C151" t="n">
+        <v>0</v>
+      </c>
+      <c r="D151" t="n">
+        <v>0</v>
+      </c>
+      <c r="E151" t="n">
+        <v>0</v>
+      </c>
+      <c r="F151" t="n">
+        <v>0</v>
+      </c>
+      <c r="G151" t="n">
+        <v>0</v>
+      </c>
+      <c r="H151" t="n">
+        <v>0</v>
+      </c>
+      <c r="I151" t="n">
+        <v>0</v>
+      </c>
+      <c r="J151" t="n">
+        <v>0</v>
+      </c>
+      <c r="K151" t="n">
+        <v>0</v>
+      </c>
+      <c r="L151" t="n">
+        <v>0</v>
+      </c>
+      <c r="M151" t="n">
+        <v>0</v>
+      </c>
+      <c r="N151" t="n">
+        <v>0</v>
+      </c>
+      <c r="O151" t="n">
+        <v>0</v>
+      </c>
+      <c r="P151" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q151" t="n">
+        <v>0</v>
+      </c>
+      <c r="R151" t="n">
+        <v>0</v>
+      </c>
+      <c r="S151" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>в том числе: автомодельный спорт</t>
+        </is>
+      </c>
+      <c r="B152" t="n">
+        <v>231</v>
+      </c>
+      <c r="C152" t="n">
+        <v>0</v>
+      </c>
+      <c r="D152" t="n">
+        <v>0</v>
+      </c>
+      <c r="E152" t="n">
+        <v>0</v>
+      </c>
+      <c r="F152" t="n">
+        <v>0</v>
+      </c>
+      <c r="G152" t="n">
+        <v>0</v>
+      </c>
+      <c r="H152" t="n">
+        <v>0</v>
+      </c>
+      <c r="I152" t="n">
+        <v>0</v>
+      </c>
+      <c r="J152" t="n">
+        <v>0</v>
+      </c>
+      <c r="K152" t="n">
+        <v>0</v>
+      </c>
+      <c r="L152" t="n">
+        <v>0</v>
+      </c>
+      <c r="M152" t="n">
+        <v>0</v>
+      </c>
+      <c r="N152" t="n">
+        <v>0</v>
+      </c>
+      <c r="O152" t="n">
+        <v>0</v>
+      </c>
+      <c r="P152" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q152" t="n">
+        <v>0</v>
+      </c>
+      <c r="R152" t="n">
+        <v>0</v>
+      </c>
+      <c r="S152" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>Айсшток</t>
+        </is>
+      </c>
+      <c r="B153" t="n">
+        <v>232</v>
+      </c>
+      <c r="C153" t="n">
+        <v>0</v>
+      </c>
+      <c r="D153" t="n">
+        <v>0</v>
+      </c>
+      <c r="E153" t="n">
+        <v>0</v>
+      </c>
+      <c r="F153" t="n">
+        <v>0</v>
+      </c>
+      <c r="G153" t="n">
+        <v>0</v>
+      </c>
+      <c r="H153" t="n">
+        <v>0</v>
+      </c>
+      <c r="I153" t="n">
+        <v>0</v>
+      </c>
+      <c r="J153" t="n">
+        <v>0</v>
+      </c>
+      <c r="K153" t="n">
+        <v>0</v>
+      </c>
+      <c r="L153" t="n">
+        <v>0</v>
+      </c>
+      <c r="M153" t="n">
+        <v>0</v>
+      </c>
+      <c r="N153" t="n">
+        <v>0</v>
+      </c>
+      <c r="O153" t="n">
+        <v>0</v>
+      </c>
+      <c r="P153" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q153" t="n">
+        <v>0</v>
+      </c>
+      <c r="R153" t="n">
+        <v>0</v>
+      </c>
+      <c r="S153" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>Водно-спасательное многоборье</t>
+        </is>
+      </c>
+      <c r="B154" t="n">
+        <v>233</v>
+      </c>
+      <c r="C154" t="n">
+        <v>0</v>
+      </c>
+      <c r="D154" t="n">
+        <v>0</v>
+      </c>
+      <c r="E154" t="n">
+        <v>0</v>
+      </c>
+      <c r="F154" t="n">
+        <v>0</v>
+      </c>
+      <c r="G154" t="n">
+        <v>0</v>
+      </c>
+      <c r="H154" t="n">
+        <v>0</v>
+      </c>
+      <c r="I154" t="n">
+        <v>0</v>
+      </c>
+      <c r="J154" t="n">
+        <v>0</v>
+      </c>
+      <c r="K154" t="n">
+        <v>0</v>
+      </c>
+      <c r="L154" t="n">
+        <v>0</v>
+      </c>
+      <c r="M154" t="n">
+        <v>0</v>
+      </c>
+      <c r="N154" t="n">
+        <v>0</v>
+      </c>
+      <c r="O154" t="n">
+        <v>0</v>
+      </c>
+      <c r="P154" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q154" t="n">
+        <v>0</v>
+      </c>
+      <c r="R154" t="n">
+        <v>0</v>
+      </c>
+      <c r="S154" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>Корфбол</t>
+        </is>
+      </c>
+      <c r="B155" t="n">
+        <v>234</v>
+      </c>
+      <c r="C155" t="n">
+        <v>0</v>
+      </c>
+      <c r="D155" t="n">
+        <v>0</v>
+      </c>
+      <c r="E155" t="n">
+        <v>0</v>
+      </c>
+      <c r="F155" t="n">
+        <v>0</v>
+      </c>
+      <c r="G155" t="n">
+        <v>0</v>
+      </c>
+      <c r="H155" t="n">
+        <v>0</v>
+      </c>
+      <c r="I155" t="n">
+        <v>0</v>
+      </c>
+      <c r="J155" t="n">
+        <v>0</v>
+      </c>
+      <c r="K155" t="n">
+        <v>0</v>
+      </c>
+      <c r="L155" t="n">
+        <v>0</v>
+      </c>
+      <c r="M155" t="n">
+        <v>0</v>
+      </c>
+      <c r="N155" t="n">
+        <v>0</v>
+      </c>
+      <c r="O155" t="n">
+        <v>0</v>
+      </c>
+      <c r="P155" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q155" t="n">
+        <v>0</v>
+      </c>
+      <c r="R155" t="n">
+        <v>0</v>
+      </c>
+      <c r="S155" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>Петанк</t>
+        </is>
+      </c>
+      <c r="B156" t="n">
+        <v>235</v>
+      </c>
+      <c r="C156" t="n">
+        <v>0</v>
+      </c>
+      <c r="D156" t="n">
+        <v>0</v>
+      </c>
+      <c r="E156" t="n">
+        <v>0</v>
+      </c>
+      <c r="F156" t="n">
+        <v>0</v>
+      </c>
+      <c r="G156" t="n">
+        <v>0</v>
+      </c>
+      <c r="H156" t="n">
+        <v>0</v>
+      </c>
+      <c r="I156" t="n">
+        <v>0</v>
+      </c>
+      <c r="J156" t="n">
+        <v>0</v>
+      </c>
+      <c r="K156" t="n">
+        <v>0</v>
+      </c>
+      <c r="L156" t="n">
+        <v>0</v>
+      </c>
+      <c r="M156" t="n">
+        <v>0</v>
+      </c>
+      <c r="N156" t="n">
+        <v>0</v>
+      </c>
+      <c r="O156" t="n">
+        <v>0</v>
+      </c>
+      <c r="P156" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q156" t="n">
+        <v>0</v>
+      </c>
+      <c r="R156" t="n">
+        <v>0</v>
+      </c>
+      <c r="S156" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>Регбол</t>
+        </is>
+      </c>
+      <c r="B157" t="n">
+        <v>236</v>
+      </c>
+      <c r="C157" t="n">
+        <v>0</v>
+      </c>
+      <c r="D157" t="n">
+        <v>0</v>
+      </c>
+      <c r="E157" t="n">
+        <v>0</v>
+      </c>
+      <c r="F157" t="n">
+        <v>0</v>
+      </c>
+      <c r="G157" t="n">
+        <v>0</v>
+      </c>
+      <c r="H157" t="n">
+        <v>0</v>
+      </c>
+      <c r="I157" t="n">
+        <v>0</v>
+      </c>
+      <c r="J157" t="n">
+        <v>0</v>
+      </c>
+      <c r="K157" t="n">
+        <v>0</v>
+      </c>
+      <c r="L157" t="n">
+        <v>0</v>
+      </c>
+      <c r="M157" t="n">
+        <v>0</v>
+      </c>
+      <c r="N157" t="n">
+        <v>0</v>
+      </c>
+      <c r="O157" t="n">
+        <v>0</v>
+      </c>
+      <c r="P157" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q157" t="n">
+        <v>0</v>
+      </c>
+      <c r="R157" t="n">
+        <v>0</v>
+      </c>
+      <c r="S157" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>Спортивная йога</t>
+        </is>
+      </c>
+      <c r="B158" t="n">
+        <v>237</v>
+      </c>
+      <c r="C158" t="n">
+        <v>0</v>
+      </c>
+      <c r="D158" t="n">
+        <v>0</v>
+      </c>
+      <c r="E158" t="n">
+        <v>0</v>
+      </c>
+      <c r="F158" t="n">
+        <v>0</v>
+      </c>
+      <c r="G158" t="n">
+        <v>0</v>
+      </c>
+      <c r="H158" t="n">
+        <v>0</v>
+      </c>
+      <c r="I158" t="n">
+        <v>0</v>
+      </c>
+      <c r="J158" t="n">
+        <v>0</v>
+      </c>
+      <c r="K158" t="n">
+        <v>0</v>
+      </c>
+      <c r="L158" t="n">
+        <v>0</v>
+      </c>
+      <c r="M158" t="n">
+        <v>0</v>
+      </c>
+      <c r="N158" t="n">
+        <v>0</v>
+      </c>
+      <c r="O158" t="n">
+        <v>0</v>
+      </c>
+      <c r="P158" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q158" t="n">
+        <v>0</v>
+      </c>
+      <c r="R158" t="n">
+        <v>0</v>
+      </c>
+      <c r="S158" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>Страйкбол</t>
+        </is>
+      </c>
+      <c r="B159" t="n">
+        <v>238</v>
+      </c>
+      <c r="C159" t="n">
+        <v>0</v>
+      </c>
+      <c r="D159" t="n">
+        <v>0</v>
+      </c>
+      <c r="E159" t="n">
+        <v>0</v>
+      </c>
+      <c r="F159" t="n">
+        <v>0</v>
+      </c>
+      <c r="G159" t="n">
+        <v>0</v>
+      </c>
+      <c r="H159" t="n">
+        <v>0</v>
+      </c>
+      <c r="I159" t="n">
+        <v>0</v>
+      </c>
+      <c r="J159" t="n">
+        <v>0</v>
+      </c>
+      <c r="K159" t="n">
+        <v>0</v>
+      </c>
+      <c r="L159" t="n">
+        <v>0</v>
+      </c>
+      <c r="M159" t="n">
+        <v>0</v>
+      </c>
+      <c r="N159" t="n">
+        <v>0</v>
+      </c>
+      <c r="O159" t="n">
+        <v>0</v>
+      </c>
+      <c r="P159" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q159" t="n">
+        <v>0</v>
+      </c>
+      <c r="R159" t="n">
+        <v>0</v>
+      </c>
+      <c r="S159" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>Флаинг диск</t>
+        </is>
+      </c>
+      <c r="B160" t="n">
+        <v>239</v>
+      </c>
+      <c r="C160" t="n">
+        <v>0</v>
+      </c>
+      <c r="D160" t="n">
+        <v>0</v>
+      </c>
+      <c r="E160" t="n">
+        <v>0</v>
+      </c>
+      <c r="F160" t="n">
+        <v>0</v>
+      </c>
+      <c r="G160" t="n">
+        <v>0</v>
+      </c>
+      <c r="H160" t="n">
+        <v>0</v>
+      </c>
+      <c r="I160" t="n">
+        <v>0</v>
+      </c>
+      <c r="J160" t="n">
+        <v>0</v>
+      </c>
+      <c r="K160" t="n">
+        <v>0</v>
+      </c>
+      <c r="L160" t="n">
+        <v>0</v>
+      </c>
+      <c r="M160" t="n">
+        <v>0</v>
+      </c>
+      <c r="N160" t="n">
+        <v>0</v>
+      </c>
+      <c r="O160" t="n">
+        <v>0</v>
+      </c>
+      <c r="P160" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q160" t="n">
+        <v>0</v>
+      </c>
+      <c r="R160" t="n">
+        <v>0</v>
+      </c>
+      <c r="S160" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>Футгольф</t>
+        </is>
+      </c>
+      <c r="B161" t="n">
+        <v>240</v>
+      </c>
+      <c r="C161" t="n">
+        <v>0</v>
+      </c>
+      <c r="D161" t="n">
+        <v>0</v>
+      </c>
+      <c r="E161" t="n">
+        <v>0</v>
+      </c>
+      <c r="F161" t="n">
+        <v>0</v>
+      </c>
+      <c r="G161" t="n">
+        <v>0</v>
+      </c>
+      <c r="H161" t="n">
+        <v>0</v>
+      </c>
+      <c r="I161" t="n">
+        <v>0</v>
+      </c>
+      <c r="J161" t="n">
+        <v>0</v>
+      </c>
+      <c r="K161" t="n">
+        <v>0</v>
+      </c>
+      <c r="L161" t="n">
+        <v>0</v>
+      </c>
+      <c r="M161" t="n">
+        <v>0</v>
+      </c>
+      <c r="N161" t="n">
+        <v>0</v>
+      </c>
+      <c r="O161" t="n">
+        <v>0</v>
+      </c>
+      <c r="P161" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q161" t="n">
+        <v>0</v>
+      </c>
+      <c r="R161" t="n">
+        <v>0</v>
+      </c>
+      <c r="S161" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>Иные виды двигательной активности (сумма строк 242-247)</t>
+        </is>
+      </c>
+      <c r="B162" t="n">
+        <v>241</v>
+      </c>
+      <c r="C162" t="n">
+        <v>0</v>
+      </c>
+      <c r="D162" t="n">
+        <v>0</v>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H162" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I162" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J162" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K162" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L162" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M162" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="N162" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O162" t="n">
+        <v>0</v>
+      </c>
+      <c r="P162" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q162" t="n">
+        <v>0</v>
+      </c>
+      <c r="R162" t="n">
+        <v>0</v>
+      </c>
+      <c r="S162" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>в том числе:хореография (танцы)</t>
+        </is>
+      </c>
+      <c r="B163" t="n">
+        <v>242</v>
+      </c>
+      <c r="C163" t="n">
+        <v>0</v>
+      </c>
+      <c r="D163" t="n">
+        <v>0</v>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G163" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H163" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I163" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J163" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K163" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L163" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M163" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="N163" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O163" t="n">
+        <v>0</v>
+      </c>
+      <c r="P163" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q163" t="n">
+        <v>0</v>
+      </c>
+      <c r="R163" t="n">
+        <v>0</v>
+      </c>
+      <c r="S163" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>вело и пешие маршруты</t>
+        </is>
+      </c>
+      <c r="B164" t="n">
+        <v>243</v>
+      </c>
+      <c r="C164" t="n">
+        <v>0</v>
+      </c>
+      <c r="D164" t="n">
+        <v>0</v>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G164" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I164" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J164" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K164" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L164" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M164" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="N164" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O164" t="n">
+        <v>0</v>
+      </c>
+      <c r="P164" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q164" t="n">
+        <v>0</v>
+      </c>
+      <c r="R164" t="n">
+        <v>0</v>
+      </c>
+      <c r="S164" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>моржевание</t>
+        </is>
+      </c>
+      <c r="B165" t="n">
+        <v>244</v>
+      </c>
+      <c r="C165" t="n">
+        <v>0</v>
+      </c>
+      <c r="D165" t="n">
+        <v>0</v>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H165" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I165" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J165" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K165" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L165" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M165" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="N165" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O165" t="n">
+        <v>0</v>
+      </c>
+      <c r="P165" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q165" t="n">
+        <v>0</v>
+      </c>
+      <c r="R165" t="n">
+        <v>0</v>
+      </c>
+      <c r="S165" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>беговелы, самокаты</t>
+        </is>
+      </c>
+      <c r="B166" t="n">
+        <v>245</v>
+      </c>
+      <c r="C166" t="n">
+        <v>0</v>
+      </c>
+      <c r="D166" t="n">
+        <v>0</v>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I166" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J166" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K166" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L166" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M166" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="N166" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O166" t="n">
+        <v>0</v>
+      </c>
+      <c r="P166" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q166" t="n">
+        <v>0</v>
+      </c>
+      <c r="R166" t="n">
+        <v>0</v>
+      </c>
+      <c r="S166" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>крикет</t>
+        </is>
+      </c>
+      <c r="B167" t="n">
+        <v>246</v>
+      </c>
+      <c r="C167" t="n">
+        <v>0</v>
+      </c>
+      <c r="D167" t="n">
+        <v>0</v>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G167" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H167" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I167" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J167" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K167" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L167" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M167" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="N167" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O167" t="n">
+        <v>0</v>
+      </c>
+      <c r="P167" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q167" t="n">
+        <v>0</v>
+      </c>
+      <c r="R167" t="n">
+        <v>0</v>
+      </c>
+      <c r="S167" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>крокет</t>
+        </is>
+      </c>
+      <c r="B168" t="n">
+        <v>247</v>
+      </c>
+      <c r="C168" t="n">
+        <v>0</v>
+      </c>
+      <c r="D168" t="n">
+        <v>0</v>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G168" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H168" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I168" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J168" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K168" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L168" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M168" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="N168" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O168" t="n">
+        <v>0</v>
+      </c>
+      <c r="P168" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q168" t="n">
+        <v>0</v>
+      </c>
+      <c r="R168" t="n">
+        <v>0</v>
+      </c>
+      <c r="S168" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>Другие</t>
+        </is>
+      </c>
+      <c r="B169" t="n">
+        <v>248</v>
+      </c>
+      <c r="C169" t="n">
+        <v>229</v>
+      </c>
+      <c r="D169" t="n">
+        <v>12</v>
+      </c>
+      <c r="E169" t="n">
+        <v>0</v>
+      </c>
+      <c r="F169" t="n">
+        <v>0</v>
+      </c>
+      <c r="G169" t="n">
+        <v>0</v>
+      </c>
+      <c r="H169" t="n">
+        <v>0</v>
+      </c>
+      <c r="I169" t="n">
+        <v>0</v>
+      </c>
+      <c r="J169" t="n">
+        <v>0</v>
+      </c>
+      <c r="K169" t="n">
+        <v>0</v>
+      </c>
+      <c r="L169" t="n">
+        <v>0</v>
+      </c>
+      <c r="M169" t="n">
+        <v>0</v>
+      </c>
+      <c r="N169" t="n">
+        <v>0</v>
+      </c>
+      <c r="O169" t="n">
+        <v>0</v>
+      </c>
+      <c r="P169" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q169" t="n">
+        <v>0</v>
+      </c>
+      <c r="R169" t="n">
+        <v>0</v>
+      </c>
+      <c r="S169" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -15875,7 +19919,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>36</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>
@@ -18200,7 +22244,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18219,11 +22263,6 @@
           <t>Всего</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Всего.1</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -18233,7 +22272,6 @@
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -18247,7 +22285,6 @@
       <c r="C3" t="n">
         <v>0</v>
       </c>
-      <c r="D3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -18261,7 +22298,6 @@
       <c r="C4" t="n">
         <v>0</v>
       </c>
-      <c r="D4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -18275,7 +22311,6 @@
       <c r="C5" t="n">
         <v>0</v>
       </c>
-      <c r="D5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -18289,7 +22324,6 @@
       <c r="C6" t="n">
         <v>0</v>
       </c>
-      <c r="D6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -18301,9 +22335,8 @@
         <v>272</v>
       </c>
       <c r="C7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D7" t="inlineStr"/>
+        <v>49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -18315,9 +22348,8 @@
         <v>273</v>
       </c>
       <c r="C8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D8" t="inlineStr"/>
+        <v>6</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -18329,9 +22361,8 @@
         <v>274</v>
       </c>
       <c r="C9" t="n">
-        <v>0</v>
-      </c>
-      <c r="D9" t="inlineStr"/>
+        <v>3</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -18345,7 +22376,6 @@
       <c r="C10" t="n">
         <v>0</v>
       </c>
-      <c r="D10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -18359,7 +22389,6 @@
       <c r="C11" t="n">
         <v>0</v>
       </c>
-      <c r="D11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -18373,7 +22402,6 @@
       <c r="C12" t="n">
         <v>0</v>
       </c>
-      <c r="D12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -18387,7 +22415,6 @@
       <c r="C13" t="n">
         <v>0</v>
       </c>
-      <c r="D13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -18401,7 +22428,6 @@
       <c r="C14" t="n">
         <v>0</v>
       </c>
-      <c r="D14" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -18436,7 +22462,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>36</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3">
@@ -18446,7 +22472,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>36</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4">
@@ -18488,7 +22514,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>85.03</v>
+        <v>127.54</v>
       </c>
     </row>
   </sheetData>
@@ -18502,7 +22528,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C37"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18879,186 +22905,6 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Присвоено спортивных званий - всего (сумма строк 269-271)</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Всего</t>
-        </is>
-      </c>
-      <c r="C26" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>в том числе: - мастер спорта</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Всего</t>
-        </is>
-      </c>
-      <c r="C27" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>-мастер спорта международного класса и Гроссмейстер России</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Всего</t>
-        </is>
-      </c>
-      <c r="C28" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>- заслуженный мастер спорта</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Всего</t>
-        </is>
-      </c>
-      <c r="C29" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>Присвоено спортивных разрядов</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Всего</t>
-        </is>
-      </c>
-      <c r="C30" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>из них: - кандидат в мастера спорта</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>Всего</t>
-        </is>
-      </c>
-      <c r="C31" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>- I разряд</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>Всего</t>
-        </is>
-      </c>
-      <c r="C32" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>Присвоено званий – заслуженный тренер России</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>Всего</t>
-        </is>
-      </c>
-      <c r="C33" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>Присвоено званий – заслуженный работник физической культуры Российской Федерации</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>Всего</t>
-        </is>
-      </c>
-      <c r="C34" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>Присуждены другие государственные почетные звания и награды</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>Всего</t>
-        </is>
-      </c>
-      <c r="C35" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>Присуждены почетные звания и награды субъекта Российской Федерации</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>Всего</t>
-        </is>
-      </c>
-      <c r="C36" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>Должностное лицо,ответственное за предоставление первичных статистических данных (лицо,уполномоченное предоставлять первичные статистические данные от имени юридического лица)</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>Всего</t>
-        </is>
-      </c>
-      <c r="C37" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>